<commit_message>
P2 step 2: near-expiry markdowns and staff discounts (DL-124..127); best deal per item
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P2.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P2.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1155,9 +1155,394 @@
       <c r="H17" s="3" t="inlineStr"/>
       <c r="I17" s="3" t="inlineStr"/>
     </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>P30</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Markdowns</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Promotions → Near-expiry markdowns: switch On (e.g. 3 days → 25%, 1 day → 50%), Save</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>'Marked down now' lists perishable lots inside the window with their %</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr"/>
+      <c r="I18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>P31</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Markdowns</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Ring up a perishable product with a lot expiring within the window</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>The line shows 'Near expiry 25% off' (or 50%) and the saving</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>P32</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Markdowns</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Phone + till</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Receive 2 more of it expiring tomorrow; ring up 3</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>2 at 50% (they sell first), 1 at 25%</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="3" t="inlineStr"/>
+      <c r="I20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>P33</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Markdowns</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>A minute later: Labels</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Near-expiry stickers on the batch, one per item, showing the marked-down price</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>P34</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Markdowns</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>A product with both a deal and a markdown</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>The customer gets whichever saves more, not both</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+      <c r="H22" s="3" t="inlineStr"/>
+      <c r="I22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>P35</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Staff discount</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Promotions → Staff discount: On, 10%, $100 a month; leave out a category; Save</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Saved; the till shows 'Staff sale'</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>P36</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Staff discount</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Ring up items, Staff sale → pick a staff member → their PIN</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>10% off each eligible item; 'Staff sale: name · $x off · $y left this month'; not on the excluded category or on items with a deal</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+      <c r="H24" s="3" t="inlineStr"/>
+      <c r="I24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>P37</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Staff discount</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Pay; look at the receipt</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>'Staff discount' under the items and 'Staff purchase: name'</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>P38</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Staff discount</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Staff sale with a wrong PIN</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Refused; no discount</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
+      <c r="H26" s="3" t="inlineStr"/>
+      <c r="I26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Staff discount</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Use up the monthly amount, then another staff sale</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>The discount stops at the limit; then 'has used this month's staff discount'</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>P40</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Staff discount</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Till (hub off)</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Switch the Pi off; try a staff sale</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Not available offline</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="3" t="inlineStr"/>
+      <c r="I28" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I17"/>
-  <conditionalFormatting sqref="F2:F17">
+  <autoFilter ref="A1:I28"/>
+  <conditionalFormatting sqref="F2:F28">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1172,7 +1557,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1186,7 +1571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1284,29 +1669,83 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Markdowns</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>COUNTIF(Tests!B:B,A4)</f>
+        <v/>
+      </c>
+      <c r="C4">
+        <f>COUNTIFS(Tests!B:B,A4,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D4">
+        <f>COUNTIFS(Tests!B:B,A4,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>COUNTIFS(Tests!B:B,A4,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F4">
+        <f>COUNTIFS(Tests!B:B,A4,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Staff discount</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>COUNTIF(Tests!B:B,A5)</f>
+        <v/>
+      </c>
+      <c r="C5">
+        <f>COUNTIFS(Tests!B:B,A5,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D5">
+        <f>COUNTIFS(Tests!B:B,A5,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>COUNTIFS(Tests!B:B,A5,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F5">
+        <f>COUNTIFS(Tests!B:B,A5,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B4" s="5">
-        <f>SUM(B2:B3)</f>
-        <v/>
-      </c>
-      <c r="C4" s="5">
-        <f>SUM(C2:C3)</f>
-        <v/>
-      </c>
-      <c r="D4" s="5">
-        <f>SUM(D2:D3)</f>
-        <v/>
-      </c>
-      <c r="E4" s="5">
-        <f>SUM(E2:E3)</f>
-        <v/>
-      </c>
-      <c r="F4" s="5">
-        <f>SUM(F2:F3)</f>
+      <c r="B6" s="5">
+        <f>SUM(B2:B5)</f>
+        <v/>
+      </c>
+      <c r="C6" s="5">
+        <f>SUM(C2:C5)</f>
+        <v/>
+      </c>
+      <c r="D6" s="5">
+        <f>SUM(D2:D5)</f>
+        <v/>
+      </c>
+      <c r="E6" s="5">
+        <f>SUM(E2:E5)</f>
+        <v/>
+      </c>
+      <c r="F6" s="5">
+        <f>SUM(F2:F5)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P2 step 3: customers and loyalty (DL-128..134); personal data never in the audit log
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P2.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P2.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1540,9 +1540,464 @@
       <c r="H28" s="3" t="inlineStr"/>
       <c r="I28" s="3" t="inlineStr"/>
     </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>P50</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Loyalty</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Home → Customers: the programme says Off. Set it up: your points per $1, points for $1 off, fewest points to use; switch On; Save</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Shows your values; only the owner can change them</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>P51</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Loyalty</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Sell: Customer → type a new phone number → Find → first name, tick 'Customer agreed' → Join</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>The customer is on the sale with 0 points and 'Earns N points'</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>P52</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Loyalty</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Pay; look at the receipt</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>'Loyalty: name', points earned and the balance</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr"/>
+      <c r="H31" s="3" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>P53</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Loyalty</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Next sale: Customer → the same phone (any format, e.g. +1 604...)</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Found with the points</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr"/>
+      <c r="H32" s="3" t="inlineStr"/>
+      <c r="I32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>P54</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Loyalty</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Use points (at least your minimum)</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Points used come off before tax ('Points used (N)'); points earned on what is paid; receipt shows earned, used, balance</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr"/>
+      <c r="H33" s="3" t="inlineStr"/>
+      <c r="I33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>P55</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Loyalty</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Return one item of that sale</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>The customer's points: the item's share of earned points taken back, its share of used points given back</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr"/>
+      <c r="H34" s="3" t="inlineStr"/>
+      <c r="I34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>P56</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Loyalty</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Customers → Loyalty cards → Make cards (e.g. 30) on a label sheet; print</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>A PDF of cards with the store name and a barcode each</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr"/>
+      <c r="H35" s="3" t="inlineStr"/>
+      <c r="I35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>P57</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Loyalty</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Scan a new card at Customer → Find</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Asks to join with that card; afterwards the card finds the customer</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr"/>
+      <c r="H36" s="3" t="inlineStr"/>
+      <c r="I36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>P58</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Loyalty</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>A customer → Card lost: block it; then link a new card</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>The old card no longer works; the points stay</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr"/>
+      <c r="H37" s="3" t="inlineStr"/>
+      <c r="I37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>P59</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Loyalty</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Adjust points with a reason; Merge two records of one person</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Points history shows it; the merged record is gone with its points moved</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr"/>
+      <c r="H38" s="3" t="inlineStr"/>
+      <c r="I38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>P60</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Loyalty</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Their data (download); then Delete on request</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>A file with everything held; after deleting, the name and phone are gone and the phone no longer finds them</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr"/>
+      <c r="H39" s="3" t="inlineStr"/>
+      <c r="I39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>P61</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Loyalty</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Till (hub off)</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Switch the Pi off; Customer → a member's phone; sell with points</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Found offline; points earned/used; the sale arrives with them when the Pi is back</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr"/>
+      <c r="H40" s="3" t="inlineStr"/>
+      <c r="I40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>P62</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Loyalty</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>As a cashier: Customers screen</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Find by phone or card only; no editing, no points adjusting</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr"/>
+      <c r="H41" s="3" t="inlineStr"/>
+      <c r="I41" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I28"/>
-  <conditionalFormatting sqref="F2:F28">
+  <autoFilter ref="A1:I41"/>
+  <conditionalFormatting sqref="F2:F41">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1557,7 +2012,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1571,7 +2026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1723,29 +2178,56 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Loyalty</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>COUNTIF(Tests!B:B,A6)</f>
+        <v/>
+      </c>
+      <c r="C6">
+        <f>COUNTIFS(Tests!B:B,A6,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D6">
+        <f>COUNTIFS(Tests!B:B,A6,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>COUNTIFS(Tests!B:B,A6,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F6">
+        <f>COUNTIFS(Tests!B:B,A6,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B6" s="5">
-        <f>SUM(B2:B5)</f>
-        <v/>
-      </c>
-      <c r="C6" s="5">
-        <f>SUM(C2:C5)</f>
-        <v/>
-      </c>
-      <c r="D6" s="5">
-        <f>SUM(D2:D5)</f>
-        <v/>
-      </c>
-      <c r="E6" s="5">
-        <f>SUM(E2:E5)</f>
-        <v/>
-      </c>
-      <c r="F6" s="5">
-        <f>SUM(F2:F5)</f>
+      <c r="B7" s="5">
+        <f>SUM(B2:B6)</f>
+        <v/>
+      </c>
+      <c r="C7" s="5">
+        <f>SUM(C2:C6)</f>
+        <v/>
+      </c>
+      <c r="D7" s="5">
+        <f>SUM(D2:D6)</f>
+        <v/>
+      </c>
+      <c r="E7" s="5">
+        <f>SUM(E2:E6)</f>
+        <v/>
+      </c>
+      <c r="F7" s="5">
+        <f>SUM(F2:F6)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P2 steps 4-5: promotion and loyalty reports, customer-facing display
- Reports > Promotions (FR-5.12): per deal vs the period before, lift, coupons, margin with costs.view
- Reports > Loyalty (FR-7.07): members, share of sales, points, liability in $, top customers
- Customer display (FR-3.14): display devices linked to a till, state in hub memory only;
  second-monitor window over BroadcastChannel (works offline)
- Tests step24 (23) and step25 (19); docs DL-135..138; manual checks P70-P86

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P2.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P2.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1995,9 +1995,499 @@
       <c r="H41" s="3" t="inlineStr"/>
       <c r="I41" s="3" t="inlineStr"/>
     </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>P70</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Home → Reports → Promotions; dates: this week</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Each deal used: times, sales, units, sales $, savings; margin %; 'before' = the week before</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr"/>
+      <c r="H42" s="3" t="inlineStr"/>
+      <c r="I42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>P71</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Open a deal's card</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Its products listed; 'All sales of its products' now vs before</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr"/>
+      <c r="H43" s="3" t="inlineStr"/>
+      <c r="I43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>P72</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>A sale with a coupon, then the report</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>The coupon code counted under 'Coupons used'</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr"/>
+      <c r="H44" s="3" t="inlineStr"/>
+      <c r="I44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>P73</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Reports → Loyalty</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Members, joined, bought; members' share of sales; points earned/used; points held and what they are worth in $</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>P74</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Top customers; Export</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>First names with the last 4 digits only; the export has the same</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr"/>
+      <c r="H46" s="3" t="inlineStr"/>
+      <c r="I46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>P75</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Change 'points for $1 off' in the programme; Reports → Loyalty again</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>'Worth' changes with the new value</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr"/>
+      <c r="H47" s="3" t="inlineStr"/>
+      <c r="I47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>P76</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (accountant)</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Sign in as Ana Accountant → Reports → Loyalty</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Totals and the liability, but no customer list</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr"/>
+      <c r="H48" s="3" t="inlineStr"/>
+      <c r="I48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>P80</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Tablet or phone</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Devices → Pair a new device: type 'Customer display'; open the code on the tablet</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>After approval it shows the store's name/logo and 'Welcome'; no sign-in</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr"/>
+      <c r="H49" s="3" t="inlineStr"/>
+      <c r="I49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>P81</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Devices → the display → 'Shows the sale of': pick the till</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>The till's card says 'Customer display: &lt;name&gt;'</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr"/>
+      <c r="H50" s="3" t="inlineStr"/>
+      <c r="I50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>P82</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Till + display</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Scan items, one with a deal; add a customer</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>The display shows the items, 'You save', the total and 'Hi &lt;name&gt; · points' within about a second</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr"/>
+      <c r="H51" s="3" t="inlineStr"/>
+      <c r="I51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>P83</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Till + display</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Pay cash with change</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Display: 'To pay' while paying, then 'Thank you!', the change and the savings</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr"/>
+      <c r="H52" s="3" t="inlineStr"/>
+      <c r="I52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>P84</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Till + display</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Wait 15 s (or New sale)</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>The display goes back to the logo and 'Welcome'</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr"/>
+      <c r="H53" s="3" t="inlineStr"/>
+      <c r="I53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>P85</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Laptop till</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Sell → 'Customer screen'; drag the window to a second monitor; sell</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>The window follows the sale; still works with the Pi switched off</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr"/>
+      <c r="H54" s="3" t="inlineStr"/>
+      <c r="I54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>P86</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Remove a deal line, change quantities, clear the sale</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>The display follows every change; nothing is left behind</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr"/>
+      <c r="H55" s="3" t="inlineStr"/>
+      <c r="I55" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I41"/>
-  <conditionalFormatting sqref="F2:F41">
+  <autoFilter ref="A1:I55"/>
+  <conditionalFormatting sqref="F2:F55">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2012,7 +2502,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2026,7 +2516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2205,29 +2695,83 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>COUNTIF(Tests!B:B,A7)</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>COUNTIFS(Tests!B:B,A7,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>COUNTIFS(Tests!B:B,A7,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>COUNTIFS(Tests!B:B,A7,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>COUNTIFS(Tests!B:B,A7,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>COUNTIF(Tests!B:B,A8)</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>COUNTIFS(Tests!B:B,A8,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>COUNTIFS(Tests!B:B,A8,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>COUNTIFS(Tests!B:B,A8,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>COUNTIFS(Tests!B:B,A8,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B7" s="5">
-        <f>SUM(B2:B6)</f>
-        <v/>
-      </c>
-      <c r="C7" s="5">
-        <f>SUM(C2:C6)</f>
-        <v/>
-      </c>
-      <c r="D7" s="5">
-        <f>SUM(D2:D6)</f>
-        <v/>
-      </c>
-      <c r="E7" s="5">
-        <f>SUM(E2:E6)</f>
-        <v/>
-      </c>
-      <c r="F7" s="5">
-        <f>SUM(F2:F6)</f>
+      <c r="B9" s="5">
+        <f>SUM(B2:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="5">
+        <f>SUM(C2:C8)</f>
+        <v/>
+      </c>
+      <c r="D9" s="5">
+        <f>SUM(D2:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="5">
+        <f>SUM(E2:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>SUM(F2:F8)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P2 step 6: dashboard and sales insights (DL-139, 140)
- Dashboard: attention list, today/month KPIs, 30-day chart with last year, margin by category,
  P&L month to date from Chedam's records, stock health; by permission on the hub
- Reports > Insights: weekday x hour heatmap, best/slowest sellers, sell-through, year over year
- ECharts (core parts only, lazy-loaded); tests step26 (19)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P2.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P2.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2485,9 +2485,254 @@
       <c r="H55" s="3" t="inlineStr"/>
       <c r="I55" s="3" t="inlineStr"/>
     </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>P90</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Home → Dashboard</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Needs attention first; sales today vs last week; this month vs last month; a 30-day chart; margin by category; this month's P&amp;L; stock health</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr"/>
+      <c r="H56" s="3" t="inlineStr"/>
+      <c r="I56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>P91</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Tap an attention line (e.g. Products out of stock)</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Opens the screen that deals with it</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr"/>
+      <c r="H57" s="3" t="inlineStr"/>
+      <c r="I57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>P92</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Phone (staff)</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Home → Dashboard as Sam Staff</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Attention and stock health only; no sales figures or P&amp;L</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr"/>
+      <c r="H58" s="3" t="inlineStr"/>
+      <c r="I58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>P93</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Make a sale, wait a minute</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Today's figures go up by themselves</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr"/>
+      <c r="H59" s="3" t="inlineStr"/>
+      <c r="I59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>P94</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Insights</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Reports → Insights; dates: last 30 days</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Totals vs last year; busy-times heatmap (switch Sales $ / Number of sales); best and slowest sellers; categories</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr"/>
+      <c r="H60" s="3" t="inlineStr"/>
+      <c r="I60" s="3" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>P95</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Insights</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Export best sellers to Excel</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Units, sales, margin, on hand and sell-through columns</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr"/>
+      <c r="H61" s="3" t="inlineStr"/>
+      <c r="I61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>P96</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Insights</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Phone, dark mode</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Open the dashboard and insights in dark mode</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Charts readable in dark colours</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr"/>
+      <c r="H62" s="3" t="inlineStr"/>
+      <c r="I62" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I55"/>
-  <conditionalFormatting sqref="F2:F55">
+  <autoFilter ref="A1:I62"/>
+  <conditionalFormatting sqref="F2:F62">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2502,7 +2747,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2516,7 +2761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2749,29 +2994,83 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>COUNTIF(Tests!B:B,A9)</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>COUNTIFS(Tests!B:B,A9,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>COUNTIFS(Tests!B:B,A9,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>COUNTIFS(Tests!B:B,A9,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>COUNTIFS(Tests!B:B,A9,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Insights</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>COUNTIF(Tests!B:B,A10)</f>
+        <v/>
+      </c>
+      <c r="C10">
+        <f>COUNTIFS(Tests!B:B,A10,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>COUNTIFS(Tests!B:B,A10,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>COUNTIFS(Tests!B:B,A10,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f>COUNTIFS(Tests!B:B,A10,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B9" s="5">
-        <f>SUM(B2:B8)</f>
-        <v/>
-      </c>
-      <c r="C9" s="5">
-        <f>SUM(C2:C8)</f>
-        <v/>
-      </c>
-      <c r="D9" s="5">
-        <f>SUM(D2:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="5">
-        <f>SUM(E2:E8)</f>
-        <v/>
-      </c>
-      <c r="F9" s="5">
-        <f>SUM(F2:F8)</f>
+      <c r="B11" s="5">
+        <f>SUM(B2:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="5">
+        <f>SUM(C2:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="5">
+        <f>SUM(D2:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="5">
+        <f>SUM(E2:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="5">
+        <f>SUM(F2:F10)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P2 step 7: tasks, checklists, handover notes, reminders (DL-141..143)
- Manual tasks with owner, due, priority, link; ticked by the person or a manager
- Opening/closing checklists: one run a day, who ticked what, late task; handover notes with read receipts
- Documents with expiry reminders (protected copy); wrong-storage tasks from product temperature ranges
- Dashboard attention: unread handover notes, unfinished checklists; api() sends forms (file uploads)
- Tests step27 (30); sample checklists, temperatures, licence

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P2.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P2.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2730,9 +2730,359 @@
       <c r="H62" s="3" t="inlineStr"/>
       <c r="I62" s="3" t="inlineStr"/>
     </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>P100</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Tasks</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Tasks and checklists → New task: for Cal, due in 1 hour, urgent, linked from a product</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Shown under Everyone's; Cal sees it under Mine</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr"/>
+      <c r="H63" s="3" t="inlineStr"/>
+      <c r="I63" s="3" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>P101</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Tasks</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Till (cashier)</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Cal: Done</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>Moves to Done with Cal's name and the time; a manager can Reopen</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr"/>
+      <c r="H64" s="3" t="inlineStr"/>
+      <c r="I64" s="3" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>P102</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Checklists</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Set up checklists: change Closing (add an optional item, done by 22:30)</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>Saved; shown in Checklists</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr"/>
+      <c r="H65" s="3" t="inlineStr"/>
+      <c r="I65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>P103</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Checklists</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Checklists → Opening: tick items; Finish with one required item left</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>Refused, names the item; ticking it then Finish works</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr"/>
+      <c r="H66" s="3" t="inlineStr"/>
+      <c r="I66" s="3" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>P104</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Checklists</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Phone + till</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Two people tick the same checklist</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Each tick shows who and when</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr"/>
+      <c r="H67" s="3" t="inlineStr"/>
+      <c r="I67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>P105</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Checklists</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Leave the closing checklist unfinished past its time</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>A task 'Closing not finished by …' appears; finishing it closes the task</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr"/>
+      <c r="H68" s="3" t="inlineStr"/>
+      <c r="I68" s="3" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>P106</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Handover</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Till → laptop</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Leave a handover note; sign in as someone else</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard: 'Handover notes you have not read'; Read it; the writer sees who read it</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr"/>
+      <c r="H69" s="3" t="inlineStr"/>
+      <c r="I69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>P107</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Licences and insurance → add insurance expiring in 5 days with a PDF</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>An urgent task 'expires on … (in 5 days)'; Open copy shows the PDF</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr"/>
+      <c r="H70" s="3" t="inlineStr"/>
+      <c r="I70" s="3" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>P108</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Change the expiry to next year</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>The task closes</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr"/>
+      <c r="H71" s="3" t="inlineStr"/>
+      <c r="I71" s="3" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>P109</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Product form: milk keep 0 to 4 °C; storage area Dry store</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>Within 10 minutes an urgent task 'needs 0–4 °C but is kept in Dry store'; back to Cooler closes it</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr"/>
+      <c r="H72" s="3" t="inlineStr"/>
+      <c r="I72" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I62"/>
-  <conditionalFormatting sqref="F2:F62">
+  <autoFilter ref="A1:I72"/>
+  <conditionalFormatting sqref="F2:F72">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2747,7 +3097,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2761,7 +3111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3048,29 +3398,164 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tasks</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>COUNTIF(Tests!B:B,A11)</f>
+        <v/>
+      </c>
+      <c r="C11">
+        <f>COUNTIFS(Tests!B:B,A11,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D11">
+        <f>COUNTIFS(Tests!B:B,A11,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E11">
+        <f>COUNTIFS(Tests!B:B,A11,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F11">
+        <f>COUNTIFS(Tests!B:B,A11,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Checklists</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>COUNTIF(Tests!B:B,A12)</f>
+        <v/>
+      </c>
+      <c r="C12">
+        <f>COUNTIFS(Tests!B:B,A12,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D12">
+        <f>COUNTIFS(Tests!B:B,A12,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>COUNTIFS(Tests!B:B,A12,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>COUNTIFS(Tests!B:B,A12,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Handover</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>COUNTIF(Tests!B:B,A13)</f>
+        <v/>
+      </c>
+      <c r="C13">
+        <f>COUNTIFS(Tests!B:B,A13,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D13">
+        <f>COUNTIFS(Tests!B:B,A13,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>COUNTIFS(Tests!B:B,A13,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>COUNTIFS(Tests!B:B,A13,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>COUNTIF(Tests!B:B,A14)</f>
+        <v/>
+      </c>
+      <c r="C14">
+        <f>COUNTIFS(Tests!B:B,A14,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D14">
+        <f>COUNTIFS(Tests!B:B,A14,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>COUNTIFS(Tests!B:B,A14,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F14">
+        <f>COUNTIFS(Tests!B:B,A14,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>COUNTIF(Tests!B:B,A15)</f>
+        <v/>
+      </c>
+      <c r="C15">
+        <f>COUNTIFS(Tests!B:B,A15,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D15">
+        <f>COUNTIFS(Tests!B:B,A15,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>COUNTIFS(Tests!B:B,A15,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>COUNTIFS(Tests!B:B,A15,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B11" s="5">
-        <f>SUM(B2:B10)</f>
-        <v/>
-      </c>
-      <c r="C11" s="5">
-        <f>SUM(C2:C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="5">
-        <f>SUM(D2:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="5">
-        <f>SUM(E2:E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="5">
-        <f>SUM(F2:F10)</f>
+      <c r="B16" s="5">
+        <f>SUM(B2:B15)</f>
+        <v/>
+      </c>
+      <c r="C16" s="5">
+        <f>SUM(C2:C15)</f>
+        <v/>
+      </c>
+      <c r="D16" s="5">
+        <f>SUM(D2:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="5">
+        <f>SUM(E2:E15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="5">
+        <f>SUM(F2:F15)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P2 step 8: messages and announcements (DL-144..146)
- Everyone channel, groups, one-to-one; mentions, product links, photo/PDF, reactions, read receipts
- Live delivery through PocketBase realtime, members only (collection rules); badge in the top bar
- Announcements that need confirming, with who has and has not read them
- Tests step28 (31, incl. realtime per member)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P2.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P2.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3080,9 +3080,359 @@
       <c r="H72" s="3" t="inlineStr"/>
       <c r="I72" s="3" t="inlineStr"/>
     </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>P110</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Messages</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Till + phone</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Messages → Everyone: write 'Truck at 2 pm' on the phone</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>The till's 💬 shows 1 within seconds; opening it shows the message</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr"/>
+      <c r="H73" s="3" t="inlineStr"/>
+      <c r="I73" s="3" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>P111</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Messages</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>New conversation → With one person (Cal); type @ and pick Cal; send</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>Cal's badge turns orange (mentioned); the message is highlighted for Cal</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr"/>
+      <c r="H74" s="3" t="inlineStr"/>
+      <c r="I74" s="3" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>P112</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Messages</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>Attach a photo of a shelf and link a product (🔗)</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>Photo thumbnail and the product link in the message; tapping the link opens the product</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr"/>
+      <c r="H75" s="3" t="inlineStr"/>
+      <c r="I75" s="3" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>P113</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Messages</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>Cal opens the conversation; back on the phone</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>Your message shows 'Read by Cal'</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr"/>
+      <c r="H76" s="3" t="inlineStr"/>
+      <c r="I76" s="3" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>P114</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Messages</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>React 👍; tap 👍 again</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>The reaction appears, then goes</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr"/>
+      <c r="H77" s="3" t="inlineStr"/>
+      <c r="I77" s="3" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>P115</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Messages</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>New conversation → A group 'Morning shift' with two people</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>Only those people see the group; others cannot open it</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr"/>
+      <c r="H78" s="3" t="inlineStr"/>
+      <c r="I78" s="3" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>P116</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Messages</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Remove your own message</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Shows 'Message removed' for everyone</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr"/>
+      <c r="H79" s="3" t="inlineStr"/>
+      <c r="I79" s="3" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>P117</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Messages</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Two devices, same person</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>Sign in as the same person on a phone and the laptop</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>The same conversations and unread counts on both</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr"/>
+      <c r="H80" s="3" t="inlineStr"/>
+      <c r="I80" s="3" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>P118</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Announcements</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>New announcement, 'Everyone must confirm'</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>Each person: banner on Home and 📌 in the top bar; 'I have read this' clears it</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr"/>
+      <c r="H81" s="3" t="inlineStr"/>
+      <c r="I81" s="3" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>P119</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Announcements</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>Look at the announcement after two people confirmed</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>'Read: …' and 'Not yet: …' lists; End removes it for everyone</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr"/>
+      <c r="H82" s="3" t="inlineStr"/>
+      <c r="I82" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I72"/>
-  <conditionalFormatting sqref="F2:F72">
+  <autoFilter ref="A1:I82"/>
+  <conditionalFormatting sqref="F2:F82">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3097,7 +3447,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3111,7 +3461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3533,29 +3883,83 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Messages</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>COUNTIF(Tests!B:B,A16)</f>
+        <v/>
+      </c>
+      <c r="C16">
+        <f>COUNTIFS(Tests!B:B,A16,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D16">
+        <f>COUNTIFS(Tests!B:B,A16,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E16">
+        <f>COUNTIFS(Tests!B:B,A16,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F16">
+        <f>COUNTIFS(Tests!B:B,A16,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Announcements</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>COUNTIF(Tests!B:B,A17)</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>COUNTIFS(Tests!B:B,A17,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D17">
+        <f>COUNTIFS(Tests!B:B,A17,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E17">
+        <f>COUNTIFS(Tests!B:B,A17,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F17">
+        <f>COUNTIFS(Tests!B:B,A17,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B16" s="5">
-        <f>SUM(B2:B15)</f>
-        <v/>
-      </c>
-      <c r="C16" s="5">
-        <f>SUM(C2:C15)</f>
-        <v/>
-      </c>
-      <c r="D16" s="5">
-        <f>SUM(D2:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="5">
-        <f>SUM(E2:E15)</f>
-        <v/>
-      </c>
-      <c r="F16" s="5">
-        <f>SUM(F2:F15)</f>
+      <c r="B18" s="5">
+        <f>SUM(B2:B17)</f>
+        <v/>
+      </c>
+      <c r="C18" s="5">
+        <f>SUM(C2:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="5">
+        <f>SUM(D2:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="5">
+        <f>SUM(E2:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="5">
+        <f>SUM(F2:F17)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P2 step 9: pings and the till overlay (DL-147..149)
- Pings to a device, all tills, phones, back office or everyone; templates; replies; take back
- Overlay over any screen (Sell keeps its sale): banner, or urgent full screen with a beep until confirmed
- Urgent pings unanswered after 5 minutes go to managers' devices and open a task (minute job)
- Tests step29 (19)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P2.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P2.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3430,9 +3430,219 @@
       <c r="H82" s="3" t="inlineStr"/>
       <c r="I82" s="3" t="inlineStr"/>
     </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>P120</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Pings</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Phone → till</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>📣 → To: Till 1 → 'Price check, please'</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>The till shows a banner with the text and quick replies, over the Sell screen</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr"/>
+      <c r="H83" s="3" t="inlineStr"/>
+      <c r="I83" s="3" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>P121</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Pings</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>With items in the cart: reply 'On my way'</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>The banner closes; the cart is still there; the phone shows '✓ Cal: On my way'</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr"/>
+      <c r="H84" s="3" t="inlineStr"/>
+      <c r="I84" s="3" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>P122</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Pings</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Phone → all tills</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Urgent: 'Manager to the front' to All tills</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>Every till turns red and beeps every 5 s; one till presses I'm on it: closed on all</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr"/>
+      <c r="H85" s="3" t="inlineStr"/>
+      <c r="I85" s="3" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>P123</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Pings</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Phone → till</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Urgent ping to a till; nobody answers for 5 minutes</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>It appears on the manager's device marked 'nobody answered', and an urgent task opens; confirming closes both</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr"/>
+      <c r="H86" s="3" t="inlineStr"/>
+      <c r="I86" s="3" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>P124</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>Pings</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Send a ping, then Take back</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>It disappears from the till</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr"/>
+      <c r="H87" s="3" t="inlineStr"/>
+      <c r="I87" s="3" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>P125</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>Pings</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Write your own ping to Everyone</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>Every device except the customer display and the sender gets it</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr"/>
+      <c r="H88" s="3" t="inlineStr"/>
+      <c r="I88" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I82"/>
-  <conditionalFormatting sqref="F2:F82">
+  <autoFilter ref="A1:I88"/>
+  <conditionalFormatting sqref="F2:F88">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3447,7 +3657,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3461,7 +3671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3937,29 +4147,56 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Pings</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>COUNTIF(Tests!B:B,A18)</f>
+        <v/>
+      </c>
+      <c r="C18">
+        <f>COUNTIFS(Tests!B:B,A18,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D18">
+        <f>COUNTIFS(Tests!B:B,A18,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E18">
+        <f>COUNTIFS(Tests!B:B,A18,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F18">
+        <f>COUNTIFS(Tests!B:B,A18,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B18" s="5">
-        <f>SUM(B2:B17)</f>
-        <v/>
-      </c>
-      <c r="C18" s="5">
-        <f>SUM(C2:C17)</f>
-        <v/>
-      </c>
-      <c r="D18" s="5">
-        <f>SUM(D2:D17)</f>
-        <v/>
-      </c>
-      <c r="E18" s="5">
-        <f>SUM(E2:E17)</f>
-        <v/>
-      </c>
-      <c r="F18" s="5">
-        <f>SUM(F2:F17)</f>
+      <c r="B19" s="5">
+        <f>SUM(B2:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="5">
+        <f>SUM(C2:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="5">
+        <f>SUM(D2:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="5">
+        <f>SUM(E2:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="5">
+        <f>SUM(F2:F18)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P2 step 10: inbox, end-of-day report, email fallback (DL-150..152)
- Per-person inbox (live badge): end-of-day report, urgent alerts, reports; choices per kind
- End-of-day report daily for the owner and chosen people; 'Today's report now'
- Deadlines and one-time email fallback marking (sending waits for the client IDs, P2-f)
- Tests step30 (19)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P2.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P2.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3640,9 +3640,254 @@
       <c r="H88" s="3" t="inlineStr"/>
       <c r="I88" s="3" t="inlineStr"/>
     </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>P130</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Inbox</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>📥 → Settings: add Mira to the end-of-day report; time 21:00; email by 07:30</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>Saved</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr"/>
+      <c r="H89" s="3" t="inlineStr"/>
+      <c r="I89" s="3" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>P131</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Inbox</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>Today's report now</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>📊 End of day …: sales, count, margin, payments, tills, best sellers, what to look at</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="inlineStr"/>
+      <c r="H90" s="3" t="inlineStr"/>
+      <c r="I90" s="3" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>P132</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Inbox</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Phone (Mira)</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Open the inbox</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>The same report (Mira sees margin: managers see costs); the 📥 count goes down when read</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr"/>
+      <c r="H91" s="3" t="inlineStr"/>
+      <c r="I91" s="3" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>P133</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Inbox</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Till (Cal)</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Open the inbox</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>No report (not chosen)</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G92" s="3" t="inlineStr"/>
+      <c r="H92" s="3" t="inlineStr"/>
+      <c r="I92" s="3" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>P134</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>Inbox</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Cause an urgent problem (milk kept in the dry store)</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>An alert ⚠ in the owner's and Mira's inbox</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G93" s="3" t="inlineStr"/>
+      <c r="H93" s="3" t="inlineStr"/>
+      <c r="I93" s="3" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>P135</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Inbox</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Phone (Mira)</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>Settings: switch off Urgent alerts in the app</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>No new alerts for Mira; the owner still gets them</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr"/>
+      <c r="H94" s="3" t="inlineStr"/>
+      <c r="I94" s="3" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>P136</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Inbox</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Next morning</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Leave the report unread past the email time</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>Shows 'email not connected yet' (sending comes with the Gmail/Outlook set-up)</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr"/>
+      <c r="H95" s="3" t="inlineStr"/>
+      <c r="I95" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I88"/>
-  <conditionalFormatting sqref="F2:F88">
+  <autoFilter ref="A1:I95"/>
+  <conditionalFormatting sqref="F2:F95">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3657,7 +3902,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F95" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3671,7 +3916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4174,29 +4419,56 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Inbox</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>COUNTIF(Tests!B:B,A19)</f>
+        <v/>
+      </c>
+      <c r="C19">
+        <f>COUNTIFS(Tests!B:B,A19,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D19">
+        <f>COUNTIFS(Tests!B:B,A19,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E19">
+        <f>COUNTIFS(Tests!B:B,A19,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F19">
+        <f>COUNTIFS(Tests!B:B,A19,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B19" s="5">
-        <f>SUM(B2:B18)</f>
-        <v/>
-      </c>
-      <c r="C19" s="5">
-        <f>SUM(C2:C18)</f>
-        <v/>
-      </c>
-      <c r="D19" s="5">
-        <f>SUM(D2:D18)</f>
-        <v/>
-      </c>
-      <c r="E19" s="5">
-        <f>SUM(E2:E18)</f>
-        <v/>
-      </c>
-      <c r="F19" s="5">
-        <f>SUM(F2:F18)</f>
+      <c r="B20" s="5">
+        <f>SUM(B2:B19)</f>
+        <v/>
+      </c>
+      <c r="C20" s="5">
+        <f>SUM(C2:C19)</f>
+        <v/>
+      </c>
+      <c r="D20" s="5">
+        <f>SUM(D2:D19)</f>
+        <v/>
+      </c>
+      <c r="E20" s="5">
+        <f>SUM(E2:E19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="5">
+        <f>SUM(F2:F19)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P2 step 11: help pages and training videos (DL-153)
- ? in the top bar opens the help page of the current screen; 19 pages, search, offline
- Training videos stored on the hub, added by settings managers
- Tests step31 (7)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P2.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P2.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$99</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I95"/>
+  <dimension ref="A1:I99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3885,9 +3885,149 @@
       <c r="H95" s="3" t="inlineStr"/>
       <c r="I95" s="3" t="inlineStr"/>
     </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>P140</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Help</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>On the Sell screen press ?</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>Help opens at 'Selling'; Back returns to Sell</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr"/>
+      <c r="H96" s="3" t="inlineStr"/>
+      <c r="I96" s="3" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>P141</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>Help</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>Search 'refund'</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>Returns and exchanges is found</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr"/>
+      <c r="H97" s="3" t="inlineStr"/>
+      <c r="I97" s="3" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>P142</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>Help</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Till (hub off)</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>Switch the Pi off; press ?</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>Help pages still open</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr"/>
+      <c r="H98" s="3" t="inlineStr"/>
+      <c r="I98" s="3" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>P143</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>Help</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>Add a training video (a short MP4 from a phone) to 'Opening and closing the till'</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>It plays from the Help page on a till</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G99" s="3" t="inlineStr"/>
+      <c r="H99" s="3" t="inlineStr"/>
+      <c r="I99" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I95"/>
-  <conditionalFormatting sqref="F2:F95">
+  <autoFilter ref="A1:I99"/>
+  <conditionalFormatting sqref="F2:F99">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3902,7 +4042,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F95" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3916,7 +4056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4446,29 +4586,56 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Help</t>
+        </is>
+      </c>
+      <c r="B20">
+        <f>COUNTIF(Tests!B:B,A20)</f>
+        <v/>
+      </c>
+      <c r="C20">
+        <f>COUNTIFS(Tests!B:B,A20,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D20">
+        <f>COUNTIFS(Tests!B:B,A20,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E20">
+        <f>COUNTIFS(Tests!B:B,A20,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F20">
+        <f>COUNTIFS(Tests!B:B,A20,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B20" s="5">
-        <f>SUM(B2:B19)</f>
-        <v/>
-      </c>
-      <c r="C20" s="5">
-        <f>SUM(C2:C19)</f>
-        <v/>
-      </c>
-      <c r="D20" s="5">
-        <f>SUM(D2:D19)</f>
-        <v/>
-      </c>
-      <c r="E20" s="5">
-        <f>SUM(E2:E19)</f>
-        <v/>
-      </c>
-      <c r="F20" s="5">
-        <f>SUM(F2:F19)</f>
+      <c r="B21" s="5">
+        <f>SUM(B2:B20)</f>
+        <v/>
+      </c>
+      <c r="C21" s="5">
+        <f>SUM(C2:C20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="5">
+        <f>SUM(D2:D20)</f>
+        <v/>
+      </c>
+      <c r="E21" s="5">
+        <f>SUM(E2:E20)</f>
+        <v/>
+      </c>
+      <c r="F21" s="5">
+        <f>SUM(F2:F20)</f>
         <v/>
       </c>
     </row>

</xml_diff>